<commit_message>
Funnel & virality batch: share card, units, email capture, vs-N, richer SEO
Turn the calculator into a growth loop:
- Personalized weakest-link -> app bridge + cookieless funnel analytics
- Shareable on-brand result PNG (native share sheet / download)
- Imperial/metric (lb<->kg) toggle at input edges; engine stays in kg
- Email capture (benchmark_emails) - anon-write RLS, only when Supabase configured
- "vs N athletes" live pool size via benchmark_pool_count() function
- SEO pages gain FAQ + how-to-improve + FAQPage/BreadcrumbList JSON-LD

Also folds in prior uncommitted work: recalibration job, pool stats,
operator standards refresh, and the programmatic SEO generator.

Build clean (42 SEO pages), 98/98 tests pass. Migration 0002 not yet applied;
not pushed, not deployed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_Operator_Standards.xlsx
+++ b/config/standards/TPF_Operator_Standards.xlsx
@@ -2479,7 +2479,7 @@
         <v>swimming</v>
       </c>
       <c r="D54" t="str">
-        <v>500 m swim</v>
+        <v>500 yd swim</v>
       </c>
       <c r="E54" t="str">
         <v>sec</v>
@@ -3087,7 +3087,7 @@
         <v>swimming</v>
       </c>
       <c r="D70" t="str">
-        <v>500 m swim</v>
+        <v>500 yd swim</v>
       </c>
       <c r="E70" t="str">
         <v>sec</v>
@@ -7379,7 +7379,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7832,9 +7832,214 @@
         <v>100</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>US</v>
+      </c>
+      <c r="B12" t="str">
+        <v>US Police PFT</v>
+      </c>
+      <c r="C12">
+        <v>35</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>30</v>
+      </c>
+      <c r="I12">
+        <v>20</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>15</v>
+      </c>
+      <c r="M12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>US</v>
+      </c>
+      <c r="B13" t="str">
+        <v>US SWAT</v>
+      </c>
+      <c r="C13">
+        <v>20</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>15</v>
+      </c>
+      <c r="G13">
+        <v>10</v>
+      </c>
+      <c r="H13">
+        <v>20</v>
+      </c>
+      <c r="I13">
+        <v>10</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>10</v>
+      </c>
+      <c r="L13">
+        <v>15</v>
+      </c>
+      <c r="M13">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>UK</v>
+      </c>
+      <c r="B14" t="str">
+        <v>UK Police JRFT</v>
+      </c>
+      <c r="C14">
+        <v>50</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>50</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>UK</v>
+      </c>
+      <c r="B15" t="str">
+        <v>UK ARU / SCO19</v>
+      </c>
+      <c r="C15">
+        <v>40</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>35</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>25</v>
+      </c>
+      <c r="M15">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>US</v>
+      </c>
+      <c r="B16" t="str">
+        <v>US Army Ranger RASP (Entry)</v>
+      </c>
+      <c r="C16">
+        <v>20</v>
+      </c>
+      <c r="D16">
+        <v>25</v>
+      </c>
+      <c r="E16">
+        <v>15</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>25</v>
+      </c>
+      <c r="I16">
+        <v>15</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>